<commit_message>
Custo por projeto: menus suspensos com lista literal na célula
Nome definido na validação não sobrevive à importação do Google Sheets de
forma confiável — foi por isso que os menus continuaram sem aparecer. A lista
passa a ser gravada dentro da própria validação, que é a forma que Excel de
mesa, Excel online, Excel do celular, LibreOffice e Google Sheets desenham.

- helper literal() valida vírgula, aspas e o limite de 255 caracteres
- TESTE 10 reescrito: confere lista literal, conteúdo item a item, tamanho,
  setinha visível e célula em branco aceita
- 329 verificações, 0 falhas

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K1S8HPUyosaj44kGisijyQ
</commit_message>
<xml_diff>
--- a/painel/planilhas/Valvic_Custo_por_Projeto.xlsx
+++ b/painel/planilhas/Valvic_Custo_por_Projeto.xlsx
@@ -11660,31 +11660,31 @@
   </conditionalFormatting>
   <dataValidations count="9">
     <dataValidation sqref="D43:D54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Este valor não está na lista. Você pode manter, mas os totais só somam o que estiver escrito exatamente como na aba Listas." type="list" errorStyle="warning">
-      <formula1>=EQUIPE_COMISSAO</formula1>
+      <formula1>"Deivson,Samuel,Cezar,Jackson,Jomar,Joelson,Jonathan Godoy,Terceiro / avulso"</formula1>
     </dataValidation>
     <dataValidation sqref="G43:G54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Este valor não está na lista. Você pode manter, mas os totais só somam o que estiver escrito exatamente como na aba Listas." type="list" errorStyle="warning">
-      <formula1>=EQUIPE_COMISSAO</formula1>
+      <formula1>"Deivson,Samuel,Cezar,Jackson,Jomar,Joelson,Jonathan Godoy,Terceiro / avulso"</formula1>
     </dataValidation>
     <dataValidation sqref="A66:A77" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Este valor não está na lista. Você pode manter, mas os totais só somam o que estiver escrito exatamente como na aba Listas." type="list" errorStyle="warning">
-      <formula1>=EQUIPE_COMISSAO</formula1>
+      <formula1>"Deivson,Samuel,Cezar,Jackson,Jomar,Joelson,Jonathan Godoy,Terceiro / avulso"</formula1>
     </dataValidation>
     <dataValidation sqref="B104:B115" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Este valor não está na lista. Você pode manter, mas os totais só somam o que estiver escrito exatamente como na aba Listas." type="list" errorStyle="warning">
-      <formula1>=CAUSA_RETRABALHO</formula1>
+      <formula1>"Erro de projeto,Erro de medição,Erro de produção,Erro de montagem,Falha de material,Dano no transporte,Mudança pedida pelo cliente,Falha de fornecedor,Outro"</formula1>
     </dataValidation>
     <dataValidation sqref="B120:B179" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Este valor não está na lista. Você pode manter, mas os totais só somam o que estiver escrito exatamente como na aba Listas." type="list" errorStyle="warning">
-      <formula1>=CATEGORIA_COMPRA</formula1>
+      <formula1>"MDF e MDP,Fita de borda,Ferragens,Vidros e espelhos,Esquadrias,Lâmina natural,Consumíveis,Acabamento,Serralheria,Vidraceiro,Outro terceirizado,Uber e aplicativo,Carreto e entrega,Deslocamento da equipe,Frete de material,Estacionamento e pedágio"</formula1>
     </dataValidation>
     <dataValidation sqref="G120:G179" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Este valor não está na lista. Você pode manter, mas os totais só somam o que estiver escrito exatamente como na aba Listas." type="list" errorStyle="warning">
-      <formula1>=FORMA_PAGAMENTO</formula1>
+      <formula1>"PIX,Boleto,Cartão de crédito,Cartão parcelado,Dinheiro,Transferência,Faturado 30 dias,A combinar"</formula1>
     </dataValidation>
     <dataValidation sqref="I120:I179" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Este valor não está na lista. Você pode manter, mas os totais só somam o que estiver escrito exatamente como na aba Listas." type="list" errorStyle="warning">
-      <formula1>=STATUS_COMPRA</formula1>
+      <formula1>"A comprar,Comprado (a pagar),Pago"</formula1>
     </dataValidation>
     <dataValidation sqref="D7:E7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Este valor não está na lista. Você pode manter, mas os totais só somam o que estiver escrito exatamente como na aba Listas." type="list" errorStyle="warning">
-      <formula1>=VENDEDOR</formula1>
+      <formula1>"Jonathan,Vitor,Indicação,Arquiteto parceiro,Outro"</formula1>
     </dataValidation>
     <dataValidation sqref="F9:G9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Este valor não está na lista. Você pode manter, mas os totais só somam o que estiver escrito exatamente como na aba Listas." type="list" errorStyle="warning">
-      <formula1>=EQUIPE_COMISSAO</formula1>
+      <formula1>"Deivson,Samuel,Cezar,Jackson,Jomar,Joelson,Jonathan Godoy,Terceiro / avulso"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.4" right="0.3" top="0.4" bottom="0.3" header="0.5" footer="0.5"/>
@@ -16385,31 +16385,31 @@
   </conditionalFormatting>
   <dataValidations count="9">
     <dataValidation sqref="D43:D54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Este valor não está na lista. Você pode manter, mas os totais só somam o que estiver escrito exatamente como na aba Listas." type="list" errorStyle="warning">
-      <formula1>=EQUIPE_COMISSAO</formula1>
+      <formula1>"Deivson,Samuel,Cezar,Jackson,Jomar,Joelson,Jonathan Godoy,Terceiro / avulso"</formula1>
     </dataValidation>
     <dataValidation sqref="G43:G54" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Este valor não está na lista. Você pode manter, mas os totais só somam o que estiver escrito exatamente como na aba Listas." type="list" errorStyle="warning">
-      <formula1>=EQUIPE_COMISSAO</formula1>
+      <formula1>"Deivson,Samuel,Cezar,Jackson,Jomar,Joelson,Jonathan Godoy,Terceiro / avulso"</formula1>
     </dataValidation>
     <dataValidation sqref="A66:A77" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Este valor não está na lista. Você pode manter, mas os totais só somam o que estiver escrito exatamente como na aba Listas." type="list" errorStyle="warning">
-      <formula1>=EQUIPE_COMISSAO</formula1>
+      <formula1>"Deivson,Samuel,Cezar,Jackson,Jomar,Joelson,Jonathan Godoy,Terceiro / avulso"</formula1>
     </dataValidation>
     <dataValidation sqref="B104:B115" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Este valor não está na lista. Você pode manter, mas os totais só somam o que estiver escrito exatamente como na aba Listas." type="list" errorStyle="warning">
-      <formula1>=CAUSA_RETRABALHO</formula1>
+      <formula1>"Erro de projeto,Erro de medição,Erro de produção,Erro de montagem,Falha de material,Dano no transporte,Mudança pedida pelo cliente,Falha de fornecedor,Outro"</formula1>
     </dataValidation>
     <dataValidation sqref="B120:B179" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Este valor não está na lista. Você pode manter, mas os totais só somam o que estiver escrito exatamente como na aba Listas." type="list" errorStyle="warning">
-      <formula1>=CATEGORIA_COMPRA</formula1>
+      <formula1>"MDF e MDP,Fita de borda,Ferragens,Vidros e espelhos,Esquadrias,Lâmina natural,Consumíveis,Acabamento,Serralheria,Vidraceiro,Outro terceirizado,Uber e aplicativo,Carreto e entrega,Deslocamento da equipe,Frete de material,Estacionamento e pedágio"</formula1>
     </dataValidation>
     <dataValidation sqref="G120:G179" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Este valor não está na lista. Você pode manter, mas os totais só somam o que estiver escrito exatamente como na aba Listas." type="list" errorStyle="warning">
-      <formula1>=FORMA_PAGAMENTO</formula1>
+      <formula1>"PIX,Boleto,Cartão de crédito,Cartão parcelado,Dinheiro,Transferência,Faturado 30 dias,A combinar"</formula1>
     </dataValidation>
     <dataValidation sqref="I120:I179" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Este valor não está na lista. Você pode manter, mas os totais só somam o que estiver escrito exatamente como na aba Listas." type="list" errorStyle="warning">
-      <formula1>=STATUS_COMPRA</formula1>
+      <formula1>"A comprar,Comprado (a pagar),Pago"</formula1>
     </dataValidation>
     <dataValidation sqref="D7:E7" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Este valor não está na lista. Você pode manter, mas os totais só somam o que estiver escrito exatamente como na aba Listas." type="list" errorStyle="warning">
-      <formula1>=VENDEDOR</formula1>
+      <formula1>"Jonathan,Vitor,Indicação,Arquiteto parceiro,Outro"</formula1>
     </dataValidation>
     <dataValidation sqref="F9:G9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Fora da lista" error="Este valor não está na lista. Você pode manter, mas os totais só somam o que estiver escrito exatamente como na aba Listas." type="list" errorStyle="warning">
-      <formula1>=EQUIPE_COMISSAO</formula1>
+      <formula1>"Deivson,Samuel,Cezar,Jackson,Jomar,Joelson,Jonathan Godoy,Terceiro / avulso"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.4" right="0.3" top="0.4" bottom="0.3" header="0.5" footer="0.5"/>

</xml_diff>